<commit_message>
Make e-mail item optional
</commit_message>
<xml_diff>
--- a/inst/formr/bvq-1.0.4/bvq_03_consent.xlsx
+++ b/inst/formr/bvq-1.0.4/bvq_03_consent.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="54">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -737,9 +737,6 @@
       <c r="C11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H11" s="1" t="s">
         <v>13</v>
       </c>

</xml_diff>